<commit_message>
LDR with Headilghts work! Added code for brake and turn lights as well.
</commit_message>
<xml_diff>
--- a/docs/pinout.xlsx
+++ b/docs/pinout.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dayoung\orange\BOAT\docs\mcu\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dayoung\orange\BOAT\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7939859A-0B78-460A-BB34-E9ACF1B4A01F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FFFEB4D-C2CC-470E-8D04-84AE401E79F4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7110" yWindow="3630" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1620" yWindow="720" windowWidth="28815" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="44">
   <si>
     <t>GND</t>
   </si>
@@ -139,6 +139,24 @@
   </si>
   <si>
     <t>ldr</t>
+  </si>
+  <si>
+    <t>headlight left</t>
+  </si>
+  <si>
+    <t>headlight right</t>
+  </si>
+  <si>
+    <t>brakelight left</t>
+  </si>
+  <si>
+    <t>brakelight right</t>
+  </si>
+  <si>
+    <t>turnlight left</t>
+  </si>
+  <si>
+    <t>turnlight right</t>
   </si>
 </sst>
 </file>
@@ -487,6 +505,8 @@
   <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="8.42578125" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -512,12 +532,14 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
         <v>22</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -527,6 +549,9 @@
       <c r="C4" t="s">
         <v>17</v>
       </c>
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
@@ -535,6 +560,9 @@
       <c r="C5" t="s">
         <v>18</v>
       </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
@@ -544,7 +572,7 @@
         <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -555,7 +583,7 @@
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -565,6 +593,9 @@
       <c r="C8" t="s">
         <v>21</v>
       </c>
+      <c r="D8" s="3" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
@@ -573,6 +604,9 @@
       <c r="C9" t="s">
         <v>23</v>
       </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
@@ -581,6 +615,9 @@
       <c r="C10" t="s">
         <v>24</v>
       </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
@@ -590,7 +627,7 @@
         <v>25</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -601,7 +638,7 @@
         <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>